<commit_message>
audit pass 3: fix swapped leaders and substitute share (LR4), TAM vs PZ1 statement and stale notes (LR2-3), evidence matrix and source log (LR4), decisions aligned with release plan (LR5), release classes note (LR6/LR7), rebuild
</commit_message>
<xml_diff>
--- a/ЛР4_Пять_сил_Портера/Excel/ЛР4_2_пять_сил_Портера_шаблон_TableMind.xlsx
+++ b/ЛР4_Пять_сил_Портера/Excel/ЛР4_2_пять_сил_Портера_шаблон_TableMind.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-3ab569\ЛР4_Пять_сил_Портера\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-89518d\ЛР4_Пять_сил_Портера\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A31BB35-4327-486F-80A9-FD0BEA056EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19D0058-9D89-41C4-BFF9-A1910DD1A6CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="12022" windowHeight="10972" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5 сил" sheetId="1" r:id="rId1"/>
@@ -543,9 +543,6 @@
     <t>Онлайн-сервисы независимой проверки Excel-моделей; англоязычные страны и ЕС</t>
   </si>
   <si>
-    <t>AI-помощники и встроенный Copilot дают около 96 % релевантного трафика сегмента; ручная проверка и Spreadsheet Inquire тоже доступны</t>
-  </si>
-  <si>
     <t>Специализированных игроков 5 (3-10), вместе с заменителями больше 10</t>
   </si>
   <si>
@@ -604,6 +601,9 @@
   </si>
   <si>
     <t>Ниша аудита таблиц неприоритетна для Microsoft и провайдеров LLM</t>
+  </si>
+  <si>
+    <t>Частичные конкуренты и заменители (AI-помощники, FP&amp;A-платформы, встроенный Copilot) дают около 73 % релевантного трафика сегмента; ручная проверка и Spreadsheet Inquire тоже доступны</t>
   </si>
 </sst>
 </file>
@@ -1155,71 +1155,8 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="7" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="6" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="6" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="7" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="6" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1233,20 +1170,83 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="9" fontId="12" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="12" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="7" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="7" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="6" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="6" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="6" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1658,13 +1658,13 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="66" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="62" t="s">
+      <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="62"/>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
@@ -1701,21 +1701,21 @@
       <c r="E10" s="9"/>
     </row>
     <row r="11" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="54" t="s">
+      <c r="A11" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="56" t="s">
+      <c r="C11" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="56"/>
-      <c r="E11" s="56"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
     </row>
     <row r="12" spans="1:6" s="10" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="55"/>
-      <c r="B12" s="57"/>
+      <c r="A12" s="34"/>
+      <c r="B12" s="36"/>
       <c r="C12" s="11">
         <v>3</v>
       </c>
@@ -1727,10 +1727,10 @@
       </c>
     </row>
     <row r="13" spans="1:6" s="10" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A13" s="40" t="s">
+      <c r="A13" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="39" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="14" t="s">
@@ -1744,62 +1744,62 @@
       </c>
     </row>
     <row r="14" spans="1:6" s="10" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="41"/>
-      <c r="B14" s="43"/>
+      <c r="A14" s="38"/>
+      <c r="B14" s="40"/>
       <c r="C14" s="15">
         <v>3</v>
       </c>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
       <c r="F14" s="10" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="16" customFormat="1" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="44" t="s">
+      <c r="A15" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="46">
+      <c r="B15" s="42"/>
+      <c r="C15" s="43">
         <f>C14+D14+E14</f>
         <v>3</v>
       </c>
-      <c r="D15" s="58"/>
-      <c r="E15" s="47"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="45"/>
     </row>
     <row r="16" spans="1:6" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="48" t="s">
+      <c r="A16" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="49"/>
-      <c r="C16" s="50" t="s">
+      <c r="B16" s="47"/>
+      <c r="C16" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="59"/>
-      <c r="E16" s="51"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
       <c r="F16" s="17"/>
     </row>
     <row r="17" spans="1:6" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="34" t="s">
+      <c r="B17" s="52"/>
+      <c r="C17" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="52"/>
-      <c r="E17" s="35"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="55"/>
     </row>
     <row r="18" spans="1:6" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="38" t="s">
+      <c r="B18" s="57"/>
+      <c r="C18" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="53"/>
-      <c r="E18" s="39"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="60"/>
     </row>
     <row r="20" spans="1:6" ht="21.4" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A20" s="8" t="s">
@@ -1811,21 +1811,21 @@
       <c r="E20" s="9"/>
     </row>
     <row r="21" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A21" s="54" t="s">
+      <c r="A21" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="56" t="s">
+      <c r="B21" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="56" t="s">
+      <c r="C21" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="56"/>
-      <c r="E21" s="56"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
     </row>
     <row r="22" spans="1:6" s="10" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="55"/>
-      <c r="B22" s="57"/>
+      <c r="A22" s="34"/>
+      <c r="B22" s="36"/>
       <c r="C22" s="11">
         <v>3</v>
       </c>
@@ -1837,10 +1837,10 @@
       </c>
     </row>
     <row r="23" spans="1:6" s="10" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="42" t="s">
+      <c r="B23" s="39" t="s">
         <v>25</v>
       </c>
       <c r="C23" s="14" t="s">
@@ -1854,22 +1854,22 @@
       </c>
     </row>
     <row r="24" spans="1:6" s="10" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="41"/>
-      <c r="B24" s="43"/>
+      <c r="A24" s="38"/>
+      <c r="B24" s="40"/>
       <c r="C24" s="15"/>
       <c r="D24" s="15">
         <v>2</v>
       </c>
       <c r="E24" s="15"/>
       <c r="F24" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="10" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A25" s="40" t="s">
+      <c r="A25" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="42" t="s">
+      <c r="B25" s="39" t="s">
         <v>30</v>
       </c>
       <c r="C25" s="14" t="s">
@@ -1883,22 +1883,22 @@
       </c>
     </row>
     <row r="26" spans="1:6" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A26" s="41"/>
-      <c r="B26" s="43"/>
+      <c r="A26" s="38"/>
+      <c r="B26" s="40"/>
       <c r="C26" s="15"/>
       <c r="D26" s="15">
         <v>2</v>
       </c>
       <c r="E26" s="15"/>
       <c r="F26" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="27" spans="1:6" s="10" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="42" t="s">
+      <c r="B27" s="39" t="s">
         <v>35</v>
       </c>
       <c r="C27" s="14" t="s">
@@ -1912,22 +1912,22 @@
       </c>
     </row>
     <row r="28" spans="1:6" s="10" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A28" s="41"/>
-      <c r="B28" s="43"/>
+      <c r="A28" s="38"/>
+      <c r="B28" s="40"/>
       <c r="C28" s="15"/>
       <c r="D28" s="15">
         <v>2</v>
       </c>
       <c r="E28" s="15"/>
       <c r="F28" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29" spans="1:6" s="16" customFormat="1" ht="56.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A29" s="40" t="s">
+      <c r="A29" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="39" t="s">
         <v>40</v>
       </c>
       <c r="C29" s="14" t="s">
@@ -1941,62 +1941,62 @@
       </c>
     </row>
     <row r="30" spans="1:6" s="16" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="41"/>
-      <c r="B30" s="43"/>
+      <c r="A30" s="38"/>
+      <c r="B30" s="40"/>
       <c r="C30" s="15"/>
       <c r="D30" s="15">
         <v>2</v>
       </c>
       <c r="E30" s="15"/>
       <c r="F30" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="31" spans="1:6" s="16" customFormat="1" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="44" t="s">
+      <c r="A31" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B31" s="45"/>
-      <c r="C31" s="46">
+      <c r="B31" s="42"/>
+      <c r="C31" s="43">
         <f>C24+D24+E24+E26+D26+C26+C28+D28+E28+C30+D30+E30</f>
         <v>8</v>
       </c>
-      <c r="D31" s="58"/>
-      <c r="E31" s="47"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="45"/>
     </row>
     <row r="32" spans="1:6" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="48" t="s">
+      <c r="A32" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="49"/>
-      <c r="C32" s="50" t="s">
+      <c r="B32" s="47"/>
+      <c r="C32" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="D32" s="59"/>
-      <c r="E32" s="51"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="50"/>
       <c r="F32" s="17"/>
     </row>
     <row r="33" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="B33" s="33"/>
-      <c r="C33" s="34" t="s">
+      <c r="B33" s="52"/>
+      <c r="C33" s="53" t="s">
         <v>47</v>
       </c>
-      <c r="D33" s="52"/>
-      <c r="E33" s="35"/>
+      <c r="D33" s="54"/>
+      <c r="E33" s="55"/>
     </row>
     <row r="34" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="36" t="s">
+      <c r="A34" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="B34" s="37"/>
-      <c r="C34" s="38" t="s">
+      <c r="B34" s="57"/>
+      <c r="C34" s="58" t="s">
         <v>49</v>
       </c>
-      <c r="D34" s="53"/>
-      <c r="E34" s="39"/>
+      <c r="D34" s="59"/>
+      <c r="E34" s="60"/>
     </row>
     <row r="36" spans="1:6" ht="21.4" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A36" s="8" t="s">
@@ -2008,21 +2008,21 @@
       <c r="E36" s="9"/>
     </row>
     <row r="37" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A37" s="54" t="s">
+      <c r="A37" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="56" t="s">
+      <c r="B37" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C37" s="56" t="s">
+      <c r="C37" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="35"/>
     </row>
     <row r="38" spans="1:6" s="10" customFormat="1" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="55"/>
-      <c r="B38" s="57"/>
+      <c r="A38" s="34"/>
+      <c r="B38" s="36"/>
       <c r="C38" s="11">
         <v>3</v>
       </c>
@@ -2034,10 +2034,10 @@
       </c>
     </row>
     <row r="39" spans="1:6" s="10" customFormat="1" ht="26.25" x14ac:dyDescent="0.5">
-      <c r="A39" s="40" t="s">
+      <c r="A39" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="B39" s="42" t="s">
+      <c r="B39" s="39" t="s">
         <v>52</v>
       </c>
       <c r="C39" s="14" t="s">
@@ -2051,22 +2051,22 @@
       </c>
     </row>
     <row r="40" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A40" s="41"/>
-      <c r="B40" s="43"/>
+      <c r="A40" s="38"/>
+      <c r="B40" s="40"/>
       <c r="C40" s="15"/>
       <c r="D40" s="15">
         <v>2</v>
       </c>
       <c r="E40" s="15"/>
       <c r="F40" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="41" spans="1:6" s="10" customFormat="1" ht="26.25" x14ac:dyDescent="0.5">
-      <c r="A41" s="40" t="s">
+      <c r="A41" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="42" t="s">
+      <c r="B41" s="39" t="s">
         <v>57</v>
       </c>
       <c r="C41" s="14" t="s">
@@ -2080,22 +2080,22 @@
       </c>
     </row>
     <row r="42" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A42" s="41"/>
-      <c r="B42" s="43"/>
+      <c r="A42" s="38"/>
+      <c r="B42" s="40"/>
       <c r="C42" s="15">
         <v>3</v>
       </c>
       <c r="D42" s="15"/>
       <c r="E42" s="15"/>
       <c r="F42" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="10" customFormat="1" ht="26.25" x14ac:dyDescent="0.5">
-      <c r="A43" s="40" t="s">
+      <c r="A43" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="B43" s="42" t="s">
+      <c r="B43" s="39" t="s">
         <v>62</v>
       </c>
       <c r="C43" s="14" t="s">
@@ -2109,22 +2109,22 @@
       </c>
     </row>
     <row r="44" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A44" s="41"/>
-      <c r="B44" s="43"/>
+      <c r="A44" s="38"/>
+      <c r="B44" s="40"/>
       <c r="C44" s="15"/>
       <c r="D44" s="15">
         <v>2</v>
       </c>
       <c r="E44" s="15"/>
       <c r="F44" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" spans="1:6" s="16" customFormat="1" ht="26.25" x14ac:dyDescent="0.5">
-      <c r="A45" s="40" t="s">
+      <c r="A45" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="B45" s="42" t="s">
+      <c r="B45" s="39" t="s">
         <v>67</v>
       </c>
       <c r="C45" s="14" t="s">
@@ -2138,22 +2138,22 @@
       </c>
     </row>
     <row r="46" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A46" s="41"/>
-      <c r="B46" s="43"/>
+      <c r="A46" s="38"/>
+      <c r="B46" s="40"/>
       <c r="C46" s="15"/>
       <c r="D46" s="15">
         <v>2</v>
       </c>
       <c r="E46" s="15"/>
       <c r="F46" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" spans="1:6" s="16" customFormat="1" ht="39.4" x14ac:dyDescent="0.5">
-      <c r="A47" s="40" t="s">
+      <c r="A47" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="B47" s="42" t="s">
+      <c r="B47" s="39" t="s">
         <v>72</v>
       </c>
       <c r="C47" s="14" t="s">
@@ -2167,22 +2167,22 @@
       </c>
     </row>
     <row r="48" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A48" s="41"/>
-      <c r="B48" s="43"/>
+      <c r="A48" s="38"/>
+      <c r="B48" s="40"/>
       <c r="C48" s="15"/>
       <c r="D48" s="15">
         <v>2</v>
       </c>
       <c r="E48" s="15"/>
       <c r="F48" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="49" spans="1:6" s="16" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A49" s="40" t="s">
+      <c r="A49" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="B49" s="42" t="s">
+      <c r="B49" s="39" t="s">
         <v>77</v>
       </c>
       <c r="C49" s="14" t="s">
@@ -2196,22 +2196,22 @@
       </c>
     </row>
     <row r="50" spans="1:6" s="16" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A50" s="41"/>
-      <c r="B50" s="43"/>
+      <c r="A50" s="38"/>
+      <c r="B50" s="40"/>
       <c r="C50" s="15"/>
       <c r="D50" s="15">
         <v>2</v>
       </c>
       <c r="E50" s="15"/>
       <c r="F50" s="16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="51" spans="1:6" s="16" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A51" s="40" t="s">
+      <c r="A51" s="37" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="42" t="s">
+      <c r="B51" s="39" t="s">
         <v>82</v>
       </c>
       <c r="C51" s="14" t="s">
@@ -2225,22 +2225,22 @@
       </c>
     </row>
     <row r="52" spans="1:6" s="16" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A52" s="41"/>
-      <c r="B52" s="43"/>
+      <c r="A52" s="38"/>
+      <c r="B52" s="40"/>
       <c r="C52" s="15"/>
       <c r="D52" s="15"/>
       <c r="E52" s="15">
         <v>1</v>
       </c>
       <c r="F52" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="53" spans="1:6" s="16" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A53" s="40" t="s">
+      <c r="A53" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="B53" s="42" t="s">
+      <c r="B53" s="39" t="s">
         <v>87</v>
       </c>
       <c r="C53" s="14" t="s">
@@ -2254,62 +2254,62 @@
       </c>
     </row>
     <row r="54" spans="1:6" s="16" customFormat="1" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="60"/>
-      <c r="B54" s="61"/>
+      <c r="A54" s="61"/>
+      <c r="B54" s="62"/>
       <c r="C54" s="18">
         <v>3</v>
       </c>
       <c r="D54" s="18"/>
       <c r="E54" s="18"/>
       <c r="F54" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="1:6" s="16" customFormat="1" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A55" s="44" t="s">
+      <c r="A55" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B55" s="45"/>
-      <c r="C55" s="46">
+      <c r="B55" s="42"/>
+      <c r="C55" s="43">
         <f>C40+D40+E40+E42+D42+C42+C44+D44+E44+E46+D46+C46+C48+D48+E48+E50+D50+C50+C52+D52+E52+C54+D54+E54</f>
         <v>17</v>
       </c>
-      <c r="D55" s="58"/>
-      <c r="E55" s="47"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="45"/>
     </row>
     <row r="56" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A56" s="48" t="s">
+      <c r="A56" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B56" s="49"/>
-      <c r="C56" s="50" t="s">
+      <c r="B56" s="47"/>
+      <c r="C56" s="48" t="s">
         <v>92</v>
       </c>
-      <c r="D56" s="59"/>
-      <c r="E56" s="51"/>
+      <c r="D56" s="49"/>
+      <c r="E56" s="50"/>
       <c r="F56" s="17"/>
     </row>
     <row r="57" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A57" s="32" t="s">
+      <c r="A57" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="B57" s="33"/>
-      <c r="C57" s="34" t="s">
+      <c r="B57" s="52"/>
+      <c r="C57" s="53" t="s">
         <v>94</v>
       </c>
-      <c r="D57" s="52"/>
-      <c r="E57" s="35"/>
+      <c r="D57" s="54"/>
+      <c r="E57" s="55"/>
     </row>
     <row r="58" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A58" s="36" t="s">
+      <c r="A58" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="B58" s="37"/>
-      <c r="C58" s="38" t="s">
+      <c r="B58" s="57"/>
+      <c r="C58" s="58" t="s">
         <v>96</v>
       </c>
-      <c r="D58" s="53"/>
-      <c r="E58" s="39"/>
+      <c r="D58" s="59"/>
+      <c r="E58" s="60"/>
     </row>
     <row r="60" spans="1:6" ht="21" x14ac:dyDescent="0.65">
       <c r="A60" s="6" t="s">
@@ -2330,21 +2330,21 @@
       <c r="E61" s="9"/>
     </row>
     <row r="62" spans="1:6" s="10" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A62" s="54" t="s">
+      <c r="A62" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B62" s="56" t="s">
+      <c r="B62" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C62" s="56" t="s">
+      <c r="C62" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="D62" s="56"/>
-      <c r="E62" s="56"/>
+      <c r="D62" s="35"/>
+      <c r="E62" s="35"/>
     </row>
     <row r="63" spans="1:6" s="10" customFormat="1" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="55"/>
-      <c r="B63" s="57"/>
+      <c r="A63" s="34"/>
+      <c r="B63" s="36"/>
       <c r="C63" s="11">
         <v>3</v>
       </c>
@@ -2356,10 +2356,10 @@
       </c>
     </row>
     <row r="64" spans="1:6" s="10" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A64" s="40" t="s">
+      <c r="A64" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="B64" s="42" t="s">
+      <c r="B64" s="39" t="s">
         <v>100</v>
       </c>
       <c r="C64" s="14" t="s">
@@ -2373,22 +2373,22 @@
       </c>
     </row>
     <row r="65" spans="1:6" s="10" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A65" s="41"/>
-      <c r="B65" s="43"/>
+      <c r="A65" s="38"/>
+      <c r="B65" s="40"/>
       <c r="C65" s="15"/>
       <c r="D65" s="15"/>
       <c r="E65" s="15">
         <v>1</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="66" spans="1:6" s="10" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A66" s="40" t="s">
+      <c r="A66" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="B66" s="42" t="s">
+      <c r="B66" s="39" t="s">
         <v>105</v>
       </c>
       <c r="C66" s="14" t="s">
@@ -2402,22 +2402,22 @@
       </c>
     </row>
     <row r="67" spans="1:6" s="10" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A67" s="41"/>
-      <c r="B67" s="43"/>
+      <c r="A67" s="38"/>
+      <c r="B67" s="40"/>
       <c r="C67" s="15">
         <v>3</v>
       </c>
       <c r="D67" s="15"/>
       <c r="E67" s="15"/>
       <c r="F67" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="68" spans="1:6" s="10" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A68" s="40" t="s">
+      <c r="A68" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="B68" s="42" t="s">
+      <c r="B68" s="39" t="s">
         <v>110</v>
       </c>
       <c r="C68" s="14" t="s">
@@ -2431,22 +2431,22 @@
       </c>
     </row>
     <row r="69" spans="1:6" s="16" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A69" s="41"/>
-      <c r="B69" s="43"/>
+      <c r="A69" s="38"/>
+      <c r="B69" s="40"/>
       <c r="C69" s="15">
         <v>3</v>
       </c>
       <c r="D69" s="15"/>
       <c r="E69" s="15"/>
       <c r="F69" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="70" spans="1:6" s="16" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A70" s="40" t="s">
+      <c r="A70" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="B70" s="42" t="s">
+      <c r="B70" s="39" t="s">
         <v>115</v>
       </c>
       <c r="C70" s="14" t="s">
@@ -2460,62 +2460,62 @@
       </c>
     </row>
     <row r="71" spans="1:6" s="16" customFormat="1" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A71" s="41"/>
-      <c r="B71" s="43"/>
+      <c r="A71" s="38"/>
+      <c r="B71" s="40"/>
       <c r="C71" s="15"/>
       <c r="D71" s="15">
         <v>2</v>
       </c>
       <c r="E71" s="15"/>
       <c r="F71" s="16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A72" s="44" t="s">
+      <c r="A72" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B72" s="45"/>
-      <c r="C72" s="46">
+      <c r="B72" s="42"/>
+      <c r="C72" s="43">
         <f>C65+D65+E65+E67+D67+C67+C69+D69+E69+C71+D71+E71</f>
         <v>9</v>
       </c>
-      <c r="D72" s="58"/>
-      <c r="E72" s="47"/>
+      <c r="D72" s="44"/>
+      <c r="E72" s="45"/>
       <c r="F72" s="17"/>
     </row>
     <row r="73" spans="1:6" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A73" s="48" t="s">
+      <c r="A73" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B73" s="49"/>
-      <c r="C73" s="50" t="s">
+      <c r="B73" s="47"/>
+      <c r="C73" s="48" t="s">
         <v>119</v>
       </c>
-      <c r="D73" s="59"/>
-      <c r="E73" s="51"/>
+      <c r="D73" s="49"/>
+      <c r="E73" s="50"/>
     </row>
     <row r="74" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A74" s="32" t="s">
+      <c r="A74" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="B74" s="33"/>
-      <c r="C74" s="34" t="s">
+      <c r="B74" s="52"/>
+      <c r="C74" s="53" t="s">
         <v>120</v>
       </c>
-      <c r="D74" s="52"/>
-      <c r="E74" s="35"/>
+      <c r="D74" s="54"/>
+      <c r="E74" s="55"/>
     </row>
     <row r="75" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A75" s="36" t="s">
+      <c r="A75" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="B75" s="37"/>
-      <c r="C75" s="38" t="s">
+      <c r="B75" s="57"/>
+      <c r="C75" s="58" t="s">
         <v>121</v>
       </c>
-      <c r="D75" s="53"/>
-      <c r="E75" s="39"/>
+      <c r="D75" s="59"/>
+      <c r="E75" s="60"/>
     </row>
     <row r="77" spans="1:6" s="10" customFormat="1" ht="21.4" thickBot="1" x14ac:dyDescent="0.7">
       <c r="A77" s="6" t="s">
@@ -2527,10 +2527,10 @@
       <c r="E77" s="20"/>
     </row>
     <row r="78" spans="1:6" s="10" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A78" s="54" t="s">
+      <c r="A78" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="B78" s="56" t="s">
+      <c r="B78" s="35" t="s">
         <v>9</v>
       </c>
       <c r="C78" s="21" t="s">
@@ -2539,8 +2539,8 @@
       <c r="D78" s="21"/>
     </row>
     <row r="79" spans="1:6" s="10" customFormat="1" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A79" s="55"/>
-      <c r="B79" s="57"/>
+      <c r="A79" s="34"/>
+      <c r="B79" s="36"/>
       <c r="C79" s="12">
         <v>2</v>
       </c>
@@ -2549,10 +2549,10 @@
       </c>
     </row>
     <row r="80" spans="1:6" s="10" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A80" s="40" t="s">
+      <c r="A80" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="B80" s="42" t="s">
+      <c r="B80" s="39" t="s">
         <v>124</v>
       </c>
       <c r="C80" s="14" t="s">
@@ -2563,21 +2563,21 @@
       </c>
     </row>
     <row r="81" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A81" s="41"/>
-      <c r="B81" s="43"/>
+      <c r="A81" s="38"/>
+      <c r="B81" s="40"/>
       <c r="C81" s="15">
         <v>2</v>
       </c>
       <c r="D81" s="15"/>
       <c r="F81" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="82" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A82" s="40" t="s">
+      <c r="A82" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="B82" s="42" t="s">
+      <c r="B82" s="39" t="s">
         <v>128</v>
       </c>
       <c r="C82" s="14" t="s">
@@ -2588,21 +2588,21 @@
       </c>
     </row>
     <row r="83" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A83" s="41"/>
-      <c r="B83" s="43"/>
+      <c r="A83" s="38"/>
+      <c r="B83" s="40"/>
       <c r="C83" s="15"/>
       <c r="D83" s="15">
         <v>1</v>
       </c>
       <c r="F83" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="84" spans="1:6" s="10" customFormat="1" ht="39.4" x14ac:dyDescent="0.5">
-      <c r="A84" s="40" t="s">
+      <c r="A84" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="B84" s="42" t="s">
+      <c r="B84" s="39" t="s">
         <v>132</v>
       </c>
       <c r="C84" s="14" t="s">
@@ -2613,21 +2613,21 @@
       </c>
     </row>
     <row r="85" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A85" s="41"/>
-      <c r="B85" s="43"/>
+      <c r="A85" s="38"/>
+      <c r="B85" s="40"/>
       <c r="C85" s="15"/>
       <c r="D85" s="15">
         <v>1</v>
       </c>
       <c r="F85" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="86" spans="1:6" s="16" customFormat="1" ht="26.25" x14ac:dyDescent="0.5">
-      <c r="A86" s="40" t="s">
+      <c r="A86" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="B86" s="42" t="s">
+      <c r="B86" s="39" t="s">
         <v>136</v>
       </c>
       <c r="C86" s="14" t="s">
@@ -2638,66 +2638,138 @@
       </c>
     </row>
     <row r="87" spans="1:6" s="16" customFormat="1" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A87" s="41"/>
-      <c r="B87" s="43"/>
+      <c r="A87" s="38"/>
+      <c r="B87" s="40"/>
       <c r="C87" s="15">
         <v>2</v>
       </c>
       <c r="D87" s="15"/>
       <c r="F87" s="16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="23.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A88" s="44" t="s">
+      <c r="A88" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B88" s="45"/>
-      <c r="C88" s="46">
+      <c r="B88" s="42"/>
+      <c r="C88" s="43">
         <f>(D81+D83+D85+D87+C81+C83+C85+C87)</f>
         <v>6</v>
       </c>
-      <c r="D88" s="47"/>
+      <c r="D88" s="45"/>
       <c r="E88" s="17"/>
     </row>
     <row r="89" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A89" s="48" t="s">
+      <c r="A89" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B89" s="49"/>
-      <c r="C89" s="50" t="s">
+      <c r="B89" s="47"/>
+      <c r="C89" s="48" t="s">
         <v>139</v>
       </c>
-      <c r="D89" s="51"/>
+      <c r="D89" s="50"/>
     </row>
     <row r="90" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A90" s="32" t="s">
+      <c r="A90" s="51" t="s">
         <v>140</v>
       </c>
-      <c r="B90" s="33"/>
-      <c r="C90" s="34" t="s">
+      <c r="B90" s="52"/>
+      <c r="C90" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="D90" s="35"/>
+      <c r="D90" s="55"/>
     </row>
     <row r="91" spans="1:6" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A91" s="36" t="s">
+      <c r="A91" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="B91" s="37"/>
-      <c r="C91" s="38" t="s">
+      <c r="B91" s="57"/>
+      <c r="C91" s="58" t="s">
         <v>143</v>
       </c>
-      <c r="D91" s="39"/>
+      <c r="D91" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="97">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="C90:D90"/>
+    <mergeCell ref="A91:B91"/>
+    <mergeCell ref="C91:D91"/>
+    <mergeCell ref="A86:A87"/>
+    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="C88:D88"/>
+    <mergeCell ref="A89:B89"/>
+    <mergeCell ref="C89:D89"/>
+    <mergeCell ref="A80:A81"/>
+    <mergeCell ref="B80:B81"/>
+    <mergeCell ref="A82:A83"/>
+    <mergeCell ref="B82:B83"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="A70:A71"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="A62:A63"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B29:B30"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="A15:B15"/>
@@ -2711,84 +2783,12 @@
     <mergeCell ref="A21:A22"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="A62:A63"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="A70:A71"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="C74:E74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="A80:A81"/>
-    <mergeCell ref="B80:B81"/>
-    <mergeCell ref="A82:A83"/>
-    <mergeCell ref="B82:B83"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="C90:D90"/>
-    <mergeCell ref="A91:B91"/>
-    <mergeCell ref="C91:D91"/>
-    <mergeCell ref="A86:A87"/>
-    <mergeCell ref="B86:B87"/>
-    <mergeCell ref="A88:B88"/>
-    <mergeCell ref="C88:D88"/>
-    <mergeCell ref="A89:B89"/>
-    <mergeCell ref="C89:D89"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="Читать теоретическую основу модели пяти сил конкуренции Макйла Портера" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>